<commit_message>
#215 - enrollment rate calculator
</commit_message>
<xml_diff>
--- a/data/enrollment/K-12 Enrollment by Age Group and Grade.xlsx
+++ b/data/enrollment/K-12 Enrollment by Age Group and Grade.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gsc\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sandag-my.sharepoint.com/personal/gsc_sandag_org/Documents/VSCode Projects/Python/Cohort-Component-Model/data/enrollment/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{5B2A16D7-01AF-44D1-8B8D-28762AD3B066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4845" yWindow="1275" windowWidth="21600" windowHeight="11295" xr2:uid="{A9FF0633-5D90-42FE-A720-036AEBF9BB82}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A9FF0633-5D90-42FE-A720-036AEBF9BB82}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="1" r:id="rId1"/>

</xml_diff>